<commit_message>
chore(samples): DAILY/BUSINESS/OTHER 소득구분 샘플 세트 추가
이지원천 업로드 검증용으로 일용/사업/기타소득 각 1명씩 들어 있는 마스터·
급여대장 xlsx 를 samples/999-99-99998/ 아래 두고, clients.xlsx 에도 해당
사업자번호(999-99-99998 "(주)소득구분샘플") 를 추가한다. 급여대장 22컬럼
표준을 따르되 4대보험은 0, 소득세·지방세만 소득구분별 세율로 산출.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/clients.xlsx
+++ b/samples/clients.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -677,6 +677,43 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>999-99-99998</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>(주)소득구분샘플</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>정샘플</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>02-999-9998</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>test@sample.co.kr</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>테스트샘플</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>법인</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>